<commit_message>
bench-assets: sync full canonical 88-task training-variant set
bench-assets/tasks-train/ was at an early 36-task snapshot; sync from the
current canonical state (which is what scripts/sync_tasks_train.sh mirrors
into Benchmarks/skillsbench/tasks-train/ at install time). Net change:

  - 52 new task variant dirs that were missing from the OSS snapshot
  - 70 existing tasks updated (Dockerfile pin bumps, variant data
    regeneration, instruction.md tweaks, test_outputs.py updates)
  - .strategy markers carried over from the variant generator

Together with the previous commit's skills/ removal, bench-assets/ now
contains exactly the 88 task variants the agent explores on, with no
curated-skill leakage.
</commit_message>
<xml_diff>
--- a/bench-assets/tasks-train/invoice-fraud-detection/environment/vendors.xlsx
+++ b/bench-assets/tasks-train/invoice-fraud-detection/environment/vendors.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Vendors" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,1078 +429,1367 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>account</t>
+          <t>iban</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>E001</t>
+          <t>VT0001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Employee 1</t>
+          <t>Acme Co.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ACCT000001</t>
+          <t>CH930076201100000001</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>E002</t>
+          <t>VT0002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Employee 2</t>
+          <t>Beacon Inc.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ACCT000002</t>
+          <t>CH930076201100000002</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>E003</t>
+          <t>VT0003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Employee 3</t>
+          <t>Crestwood Solutions</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ACCT000003</t>
+          <t>CH930076201100000003</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>E004</t>
+          <t>VT0004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Employee 4</t>
+          <t>Delphi Co.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ACCT000004</t>
+          <t>CH930076201100000004</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>E005</t>
+          <t>VT0005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Employee 5</t>
+          <t>Everest Corp</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ACCT000005</t>
+          <t>CH930076201100000005</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>E006</t>
+          <t>VT0006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Employee 6</t>
+          <t>Fairfax Systems</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ACCT000006</t>
+          <t>CH930076201100000006</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>E007</t>
+          <t>VT0007</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Employee 7</t>
+          <t>Granite Works</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ACCT000007</t>
+          <t>CH930076201100000007</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>E008</t>
+          <t>VT0008</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Employee 8</t>
+          <t>Horizon Works</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ACCT000008</t>
+          <t>CH930076201100000008</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>E009</t>
+          <t>VT0009</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Employee 9</t>
+          <t>Ironclad LLC</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ACCT000009</t>
+          <t>CH930076201100000009</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>E010</t>
+          <t>VT0010</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Employee 10</t>
+          <t>Juniper Works</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ACCT000010</t>
+          <t>CH930076201100000010</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>E011</t>
+          <t>VT0011</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Employee 11</t>
+          <t>Keystone Industries</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ACCT000011</t>
+          <t>CH930076201100000011</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>E012</t>
+          <t>VT0012</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Employee 12</t>
+          <t>Larkspur Corp</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ACCT000012</t>
+          <t>CH930076201100000012</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>E013</t>
+          <t>VT0013</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Employee 13</t>
+          <t>Meridian Group</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ACCT000013</t>
+          <t>CH930076201100000013</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>E014</t>
+          <t>VT0014</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Employee 14</t>
+          <t>Northwind Works</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ACCT000014</t>
+          <t>CH930076201100000014</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>E015</t>
+          <t>VT0015</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Employee 15</t>
+          <t>Oakridge Inc.</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ACCT000015</t>
+          <t>CH930076201100000015</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>E016</t>
+          <t>VT0016</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Employee 16</t>
+          <t>Pioneer Holdings</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ACCT000016</t>
+          <t>CH930076201100000016</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>E017</t>
+          <t>VT0017</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Employee 17</t>
+          <t>Quartz Works</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ACCT000017</t>
+          <t>CH930076201100000017</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>E018</t>
+          <t>VT0018</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Employee 18</t>
+          <t>Redwood Ltd</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ACCT000018</t>
+          <t>CH930076201100000018</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>E019</t>
+          <t>VT0019</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Employee 19</t>
+          <t>Silverleaf Supplies</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ACCT000019</t>
+          <t>CH930076201100000019</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>E020</t>
+          <t>VT0020</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Employee 20</t>
+          <t>Tidewater Works</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ACCT000020</t>
+          <t>CH930076201100000020</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>E021</t>
+          <t>VT0021</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Employee 21</t>
+          <t>Umbra Solutions</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ACCT000021</t>
+          <t>CH930076201100000021</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>E022</t>
+          <t>VT0022</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Employee 22</t>
+          <t>Vanguard Solutions</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ACCT000022</t>
+          <t>CH930076201100000022</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>E023</t>
+          <t>VT0023</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Employee 23</t>
+          <t>Westgate Corp</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ACCT000023</t>
+          <t>CH930076201100000023</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>E024</t>
+          <t>VT0024</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Employee 24</t>
+          <t>Xenon Inc.</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ACCT000024</t>
+          <t>CH930076201100000024</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>E025</t>
+          <t>VT0025</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Employee 25</t>
+          <t>Yellowstone Ltd</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ACCT000025</t>
+          <t>CH930076201100000025</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>E026</t>
+          <t>VT0026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Employee 26</t>
+          <t>Zenith Systems</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ACCT000026</t>
+          <t>CH930076201100000026</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>E027</t>
+          <t>VT0027</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Employee 27</t>
+          <t>Alpine Supplies</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ACCT000027</t>
+          <t>CH930076201100000027</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>E028</t>
+          <t>VT0028</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Employee 28</t>
+          <t>Blackrock &amp; Associates</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ACCT000028</t>
+          <t>CH930076201100000028</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>E029</t>
+          <t>VT0029</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Employee 29</t>
+          <t>Cascade Holdings</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ACCT000029</t>
+          <t>CH930076201100000029</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>E030</t>
+          <t>VT0030</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Employee 30</t>
+          <t>Driftwood Industries</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ACCT000030</t>
+          <t>CH930076201100000030</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>E031</t>
+          <t>VT0031</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Employee 31</t>
+          <t>Emberline Partners</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ACCT000031</t>
+          <t>CH930076201100000031</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>E032</t>
+          <t>VT0032</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Employee 32</t>
+          <t>Fortis Group</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ACCT000032</t>
+          <t>CH930076201100000032</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>E033</t>
+          <t>VT0033</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Employee 33</t>
+          <t>Gryphon Ltd</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ACCT000033</t>
+          <t>CH930076201100000033</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>E034</t>
+          <t>VT0034</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Employee 34</t>
+          <t>Halcyon LLC</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ACCT000034</t>
+          <t>CH930076201100000034</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>E035</t>
+          <t>VT0035</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Employee 35</t>
+          <t>Ironwood Group</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ACCT000035</t>
+          <t>CH930076201100000035</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>E036</t>
+          <t>VT0036</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Employee 36</t>
+          <t>Jadewood Works</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ACCT000036</t>
+          <t>CH930076201100000036</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>E037</t>
+          <t>VT0037</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Employee 37</t>
+          <t>Kestrel Corp</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ACCT000037</t>
+          <t>CH930076201100000037</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>E038</t>
+          <t>VT0038</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Employee 38</t>
+          <t>Lumina Ltd</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ACCT000038</t>
+          <t>CH930076201100000038</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>E039</t>
+          <t>VT0039</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Employee 39</t>
+          <t>Marble Solutions</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ACCT000039</t>
+          <t>CH930076201100000039</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>E040</t>
+          <t>VT0040</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Employee 40</t>
+          <t>Nimbus &amp; Associates</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ACCT000040</t>
+          <t>CH930076201100000040</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>E041</t>
+          <t>VT0041</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Employee 41</t>
+          <t>Obsidian Works</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ACCT000041</t>
+          <t>CH930076201100000041</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>E042</t>
+          <t>VT0042</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Employee 42</t>
+          <t>Prairie Supplies</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ACCT000042</t>
+          <t>CH930076201100000042</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>E043</t>
+          <t>VT0043</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Employee 43</t>
+          <t>Quorum Holdings</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ACCT000043</t>
+          <t>CH930076201100000043</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>E044</t>
+          <t>VT0044</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Employee 44</t>
+          <t>Riverstone Co.</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ACCT000044</t>
+          <t>CH930076201100000044</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>E045</t>
+          <t>VT0045</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Employee 45</t>
+          <t>Solstice Inc.</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ACCT000045</t>
+          <t>CH930076201100000045</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>E046</t>
+          <t>VT0046</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Employee 46</t>
+          <t>Thornfield Systems</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ACCT000046</t>
+          <t>CH930076201100000046</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>E047</t>
+          <t>VT0047</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Employee 47</t>
+          <t>Uplift Group</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ACCT000047</t>
+          <t>CH930076201100000047</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>E048</t>
+          <t>VT0048</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Employee 48</t>
+          <t>Vertex Systems</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ACCT000048</t>
+          <t>CH930076201100000048</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>E049</t>
+          <t>VT0049</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Employee 49</t>
+          <t>Willowbrook Ltd</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ACCT000049</t>
+          <t>CH930076201100000049</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>E050</t>
+          <t>VT0050</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Employee 50</t>
+          <t>Ximen Industries</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ACCT000050</t>
+          <t>CH930076201100000050</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>E051</t>
+          <t>VT0051</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Employee 51</t>
+          <t>Yarrow &amp; Associates</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ACCT000051</t>
+          <t>CH930076201100000051</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>E052</t>
+          <t>VT0052</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Employee 52</t>
+          <t>Zircon Holdings</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ACCT000052</t>
+          <t>CH930076201100000052</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>E053</t>
+          <t>VT0053</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Employee 53</t>
+          <t>Ashcroft LLC</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ACCT000053</t>
+          <t>CH930076201100000053</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>E054</t>
+          <t>VT0054</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Employee 54</t>
+          <t>Briarwood Holdings</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ACCT000054</t>
+          <t>CH930076201100000054</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>E055</t>
+          <t>VT0055</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Employee 55</t>
+          <t>Copperfield Solutions</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ACCT000055</t>
+          <t>CH930076201100000055</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>E056</t>
+          <t>VT0056</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Employee 56</t>
+          <t>Dawnstar Group</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ACCT000056</t>
+          <t>CH930076201100000056</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>E057</t>
+          <t>VT0057</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Employee 57</t>
+          <t>Elmpoint Systems</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ACCT000057</t>
+          <t>CH930076201100000057</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>E058</t>
+          <t>VT0058</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Employee 58</t>
+          <t>Foxglove LLC</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ACCT000058</t>
+          <t>CH930076201100000058</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>E059</t>
+          <t>VT0059</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Employee 59</t>
+          <t>Grayhaven Co.</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>ACCT000059</t>
+          <t>CH930076201100000059</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>E060</t>
+          <t>VT0060</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Employee 60</t>
+          <t>Hearthstone &amp; Associates</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>ACCT000060</t>
+          <t>CH930076201100000060</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>E901</t>
+          <t>VT0061</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Reliable Worker Co.</t>
+          <t>Ivywood Co.</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>ACCTSAFE901</t>
+          <t>CH930076201100000061</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>E902</t>
+          <t>VT0062</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Fuzzy Name Consulting Inc.</t>
+          <t>Jasper Supplies</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>ACCTFUZZ902</t>
+          <t>CH930076201100000062</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>E903</t>
+          <t>VT0063</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Threshold Edge LLC</t>
+          <t>Kindleberg Logistics</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>ACCTEDGE903</t>
+          <t>CH930076201100000063</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>VT0064</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Lanternwood Partners</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>CH930076201100000064</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>VT0065</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Mosswell LLC</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>CH930076201100000065</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>VT0066</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Nightfall Partners</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>CH930076201100000066</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>VT0067</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Olivebranch Holdings</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>CH930076201100000067</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>VT0068</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Patternworks Industries</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>CH930076201100000068</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>VT0069</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Quietrun LLC</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>CH930076201100000069</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>VT0070</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Roseberry &amp; Associates</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>CH930076201100000070</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>VT0071</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Sagehill Inc.</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>CH930076201100000071</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>VT0072</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Tinderwood Solutions</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>CH930076201100000072</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>VT0073</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Undertow Inc.</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>CH930076201100000073</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>VT0074</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Violetpoint Co.</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>CH930076201100000074</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>VT0075</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Whitestone LLC</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>CH930076201100000075</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>VT0076</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Xavian Works</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>CH930076201100000076</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>VT0077</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Yearwood Holdings</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>CH930076201100000077</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>VT0078</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Zephyrus Ltd</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>CH930076201100000078</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>VT0079</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Aldergate Supplies</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>CH930076201100000079</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>VT0080</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Bramblewood Solutions</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>CH930076201100000080</t>
         </is>
       </c>
     </row>

</xml_diff>